<commit_message>
some improvements in the words file
</commit_message>
<xml_diff>
--- a/data/Click Me (Geography Demo).xlsx
+++ b/data/Click Me (Geography Demo).xlsx
@@ -24,18 +24,6 @@
     <t>Canberra</t>
   </si>
   <si>
-    <t>Indonesia</t>
-  </si>
-  <si>
-    <t>Jakarta</t>
-  </si>
-  <si>
-    <t>Maldives</t>
-  </si>
-  <si>
-    <t>Male</t>
-  </si>
-  <si>
     <t>South Africa</t>
   </si>
   <si>
@@ -54,10 +42,22 @@
     <t>Reykjavik</t>
   </si>
   <si>
-    <t>Egypt</t>
-  </si>
-  <si>
-    <t>Cairo</t>
+    <t>Paris</t>
+  </si>
+  <si>
+    <t>France</t>
+  </si>
+  <si>
+    <t>Tokyo</t>
+  </si>
+  <si>
+    <t>Japan</t>
+  </si>
+  <si>
+    <t>Moscow</t>
+  </si>
+  <si>
+    <t>Russia</t>
   </si>
 </sst>
 </file>
@@ -398,61 +398,64 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.88671875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>